<commit_message>
Harnais de tests du site aligne sur la spec v1.2 et rapport filtre sur les decisions en attente (session Tests de specifications)
- site_audit.py : UT-PAGE-19 = liens produits en nouvel onglet ; IT-NAV-01/02/05/06/07 et PT-LINK-01 verifient target=_blank + noopener + noreferrer ; anciens controles marque en UT-AUX-* ; correction du shadowing rel dans PT-LINK
- build_site_full_report.py : classeur ouvert filtre sur Action souhaitee (lignes non decidees), reprise des decisions du classeur de meme nom, lignes Resolu pour la trace
- Run du 16/09 22h03 : 120 cas, 76 Pass / 6 Fail (Mineurs, inchanges) / 38 Bloques, 0 regression

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260915a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260915a.xlsx
@@ -462,14 +462,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260915a) - execute le 2026-09-15T18:38:57.278563</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="58" customHeight="1">
+          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260915a) - execute le 2026-09-16T22:03:15.249785</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>44 lignes a revoir sur 119 cas : 6 defauts (echecs, tous Mineurs) et 38 bloques. Les defauts sont en haut, puis les cas bloques (Gravite = 'Bloque' : le test n'a pas pu etre joue - la colonne 'Ce qui ne va pas' dit pourquoi et ce qu'il faut). Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 6 defauts (echecs) + 38 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur la colonne 'Action souhaitee' pour ne montrer que les lignes ou vous n'avez PAS encore demande de correction. Pour revoir tout l'historique (y compris ce que vous avez deja decide, ou les points corriges/plus detectes), enlevez le filtre de la colonne 'Action souhaitee'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,11 @@
       <c r="J48" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J48"/>
+  <autoFilter ref="A4:J48">
+    <filterColumn colId="8" hiddenButton="0" showButton="1">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Harnais et resultats de tests du site alignes v1.3/v1.4 (session Tests de specifications)
- site_audit.py : VERSION_TAG 20260915a -> 20260917a ; nouveaux controles UT-PAGE-20 (durcissement formulaire), UT-PAGE-21 + PT-INFO-04 (coordonnees et cle jamais en clair, inversees dans data-*), PT-INPUT-01 en Bloque (necessite jusqu a 5 envois reels marques TEST, accord de Lydie requis)
- Run du 17/09 : 125 cas, 6 defauts (Mineurs connus), 40 bloques, 0 regression, aucun nouveau defaut
- Classeur resultats-tests-site-web-20260917a.xlsx (reprise des decisions precedentes, trace conservee)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260915a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260915a.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A revoir" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'A revoir'!$A$4:$J$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'A revoir'!$A$4:$J$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -462,14 +462,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260915a) - execute le 2026-09-16T22:03:15.249785</t>
+          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260915a) - execute le 2026-09-17T13:54:29.612249</t>
         </is>
       </c>
     </row>
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Un seul onglet, 6 defauts (echecs) + 38 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur la colonne 'Action souhaitee' pour ne montrer que les lignes ou vous n'avez PAS encore demande de correction. Pour revoir tout l'historique (y compris ce que vous avez deja decide, ou les points corriges/plus detectes), enlevez le filtre de la colonne 'Action souhaitee'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 7 defauts (echecs) + 39 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur la colonne 'Action souhaitee' pour ne montrer que les lignes ou vous n'avez PAS encore demande de correction. Pour revoir tout l'historique (y compris ce que vous avez deja decide, ou les points corriges/plus detectes), enlevez le filtre de la colonne 'Action souhaitee'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -792,51 +792,39 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-02</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>UT-PAGE-13</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test unitaire</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>real submission FR</t>
+          <t>CSS / JS version tags</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Toi (accès ou accord requis)</t>
-        </is>
-      </c>
+          <t>index.html:css/fonts.css=20260917a; index.html:css/styles.css=20260917a; index.html:css/fusion.css=20260917a; index.html:js/script.js=20260917a; a-propos.html:css/fonts.css=20260917a; a-propos.html:css/styles.css=20260917a</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-03</t>
+          <t>IT-FORM-02</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -851,22 +839,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>real submission EN</t>
+          <t>real submission FR</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ce test n'a pas pu être joué automatiquement : il demande une action manuelle ou un accès externe. À exécuter par le testeur.</t>
+          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : reste à exécuter.</t>
+          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Cas non automatisable dans le contrôle actuel (action manuelle ou accès externe requis).</t>
+          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -880,7 +868,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>PT-CLICK-01</t>
+          <t>IT-FORM-03</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -890,27 +878,27 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test d'intégration</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Clickjacking</t>
+          <t>real submission EN</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Test de « mise en cadre » du site (clickjacking) : à confirmer dans un navigateur ; GitHub Pages ne permet pas d'ajouter l'en-tête de protection habituel.</t>
+          <t>Ce test n'a pas pu être joué automatiquement : il demande une action manuelle ou un accès externe. À exécuter par le testeur.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer en navigateur.</t>
+          <t>Aucun défaut détecté : reste à exécuter.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Clickjacking (framing) : à confirmer en navigateur ; en-têtes X-Frame-Options/CSP non modifiables sur GitHub Pages.</t>
+          <t>Cas non automatisable dans le contrôle actuel (action manuelle ou accès externe requis).</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -924,7 +912,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PT-DNS-02</t>
+          <t>PT-CLICK-01</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -939,22 +927,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Zone hygiene</t>
+          <t>Clickjacking</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
+          <t>Test de « mise en cadre » du site (clickjacking) : à confirmer dans un navigateur ; GitHub Pages ne permet pas d'ajouter l'en-tête de protection habituel.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
+          <t>Aucun défaut détecté : à confirmer en navigateur.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
+          <t>Clickjacking (framing) : à confirmer en navigateur ; en-têtes X-Frame-Options/CSP non modifiables sur GitHub Pages.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -968,7 +956,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-01</t>
+          <t>PT-DNS-02</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -983,22 +971,22 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Form abuse</t>
+          <t>Zone hygiene</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1012,7 +1000,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-02</t>
+          <t>PT-FORM-01</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1027,7 +1015,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Rate and quota</t>
+          <t>Form abuse</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1056,7 +1044,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-03</t>
+          <t>PT-FORM-02</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1071,7 +1059,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Privacy of submissions</t>
+          <t>Rate and quota</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1100,7 +1088,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PT-PRIV-01</t>
+          <t>PT-FORM-03</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1115,27 +1103,27 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>Privacy of submissions</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Vérification « zéro cookie / zéro traqueur » en conditions réelles : à confirmer dans un navigateur en naviguant sur le site en ligne.</t>
+          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer en navigation réelle.</t>
+          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Absence de cookies / traqueurs en conditions réelles : à confirmer via les outils du navigateur sur le site déployé.</t>
+          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Testeur / navigateur</t>
+          <t>Toi (accès ou accord requis)</t>
         </is>
       </c>
       <c r="I18" s="4" t="n"/>
@@ -1144,7 +1132,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-01</t>
+          <t>PT-INPUT-01</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1159,22 +1147,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Supply chain</t>
+          <t>Input validation (WSTG-INPV)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
+          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
+          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
+          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1188,7 +1176,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-02</t>
+          <t>PT-PRIV-01</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1203,27 +1191,27 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Publication integrity</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
+          <t>Vérification « zéro cookie / zéro traqueur » en conditions réelles : à confirmer dans un navigateur en naviguant sur le site en ligne.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
+          <t>Aucun défaut détecté : à confirmer en navigation réelle.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
+          <t>Absence de cookies / traqueurs en conditions réelles : à confirmer via les outils du navigateur sur le site déployé.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Testeur / navigateur</t>
         </is>
       </c>
       <c r="I20" s="4" t="n"/>
@@ -1232,7 +1220,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PT-TLS-02</t>
+          <t>PT-SUPPLY-01</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1247,27 +1235,27 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>HSTS</t>
+          <t>Supply chain</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Note complète du chiffrement HTTPS (versions, algorithmes) : se mesure avec un outil externe (SSL Labs) sur le domaine en ligne, pas dans ce contrôle automatique.</t>
+          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à mesurer sur le domaine en ligne.</t>
+          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Grade TLS complet (protocoles, ciphers) : nécessite testssl.sh / SSL Labs sur le domaine public.</t>
+          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Testeur / navigateur</t>
+          <t>Toi (accès ou accord requis)</t>
         </is>
       </c>
       <c r="I21" s="4" t="n"/>
@@ -1276,7 +1264,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-02</t>
+          <t>PT-SUPPLY-02</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1286,32 +1274,32 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>keyboard only</t>
+          <t>Publication integrity</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
+          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
+          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
+          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
+          <t>Toi (accès ou accord requis)</t>
         </is>
       </c>
       <c r="I22" s="4" t="n"/>
@@ -1320,7 +1308,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-03</t>
+          <t>PT-TLS-02</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1330,32 +1318,32 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>screen reader (NVDA) on the home</t>
+          <t>HSTS</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
+          <t>Note complète du chiffrement HTTPS (versions, algorithmes) : se mesure avec un outil externe (SSL Labs) sur le domaine en ligne, pas dans ce contrôle automatique.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
+          <t>Aucun défaut détecté : à mesurer sur le domaine en ligne.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
+          <t>Grade TLS complet (protocoles, ciphers) : nécessite testssl.sh / SSL Labs sur le domaine public.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
+          <t>Testeur / navigateur</t>
         </is>
       </c>
       <c r="I23" s="4" t="n"/>
@@ -1364,7 +1352,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-04</t>
+          <t>ST-A11Y-02</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1379,7 +1367,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>contrast and zoom</t>
+          <t>keyboard only</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1408,7 +1396,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-05</t>
+          <t>ST-A11Y-03</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1423,7 +1411,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>motion</t>
+          <t>screen reader (NVDA) on the home</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1452,7 +1440,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-02</t>
+          <t>ST-A11Y-04</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1467,7 +1455,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>same from EN</t>
+          <t>contrast and zoom</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1496,7 +1484,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-03</t>
+          <t>ST-A11Y-05</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1511,7 +1499,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>offline (devtools)</t>
+          <t>motion</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1540,7 +1528,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-04</t>
+          <t>ST-CONTACT-02</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1555,7 +1543,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>e-mail / phone links</t>
+          <t>same from EN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1584,7 +1572,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-01</t>
+          <t>ST-CONTACT-03</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1599,7 +1587,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>hero and figures band</t>
+          <t>offline (devtools)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1628,7 +1616,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-03</t>
+          <t>ST-CONTACT-04</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1643,7 +1631,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>À propos + HOME tiles</t>
+          <t>e-mail / phone links</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1672,7 +1660,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-04</t>
+          <t>ST-HOME-01</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1687,7 +1675,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Produits de santé and Expertises</t>
+          <t>hero and figures band</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1716,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-05</t>
+          <t>ST-HOME-03</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1731,7 +1719,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Secteurs, OKILYS Suite panel, Contact</t>
+          <t>À propos + HOME tiles</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1760,7 +1748,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-03</t>
+          <t>ST-HOME-04</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1775,7 +1763,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>carousel</t>
+          <t>Produits de santé and Expertises</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1804,7 +1792,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-04</t>
+          <t>ST-HOME-05</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1819,7 +1807,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>Secteurs, OKILYS Suite panel, Contact</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1848,7 +1836,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-05</t>
+          <t>ST-MOB-03</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1863,7 +1851,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>tablet 768 px</t>
+          <t>carousel</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1892,7 +1880,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ST-NAV-03</t>
+          <t>ST-MOB-04</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1907,7 +1895,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>scrollspy</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1936,7 +1924,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ST-NAV-05</t>
+          <t>ST-MOB-05</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1951,7 +1939,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>back / forward</t>
+          <t>tablet 768 px</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1980,7 +1968,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-01</t>
+          <t>ST-NAV-03</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1995,7 +1983,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>5 product pages</t>
+          <t>scrollspy</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2024,7 +2012,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-02</t>
+          <t>ST-NAV-05</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2039,7 +2027,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>7 step pages</t>
+          <t>back / forward</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2068,7 +2056,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-03</t>
+          <t>ST-PAGE-01</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2083,7 +2071,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>About page</t>
+          <t>5 product pages</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2112,7 +2100,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-04</t>
+          <t>ST-PAGE-02</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2127,7 +2115,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Réalisations and Actualités</t>
+          <t>7 step pages</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2156,7 +2144,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-06</t>
+          <t>ST-PAGE-03</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2171,7 +2159,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Legal and 404</t>
+          <t>About page</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2200,7 +2188,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ST-PERF-02</t>
+          <t>ST-PAGE-04</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -2215,7 +2203,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>fonts</t>
+          <t>Réalisations and Actualités</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2244,7 +2232,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ST-PERF-03</t>
+          <t>ST-PAGE-06</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2259,7 +2247,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>cache behaviour after a publication</t>
+          <t>Legal and 404</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2288,7 +2276,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-02</t>
+          <t>ST-PERF-02</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2303,7 +2291,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Google Rich Results test on home, About, a product page, `ctms`</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2332,7 +2320,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-03</t>
+          <t>ST-PERF-03</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2347,7 +2335,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Search Console and Bing Webmaster</t>
+          <t>cache behaviour after a publication</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2376,7 +2364,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-04</t>
+          <t>ST-SEO-02</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -2391,7 +2379,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>hreflang validator (e.g. Merkle / Sistrix) on 6 pages</t>
+          <t>Google Rich Results test on home, About, a product page, `ctms`</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2420,7 +2408,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-05</t>
+          <t>ST-SEO-03</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2435,7 +2423,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>snippet preview</t>
+          <t>Search Console and Bing Webmaster</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2461,8 +2449,96 @@
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="4" t="n"/>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ST-SEO-04</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Bloqué</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>hreflang validator (e.g. Merkle / Sistrix) on 6 pages</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="n"/>
+      <c r="J49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>ST-SEO-05</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Bloqué</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>snippet preview</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="n"/>
+      <c r="J50" s="4" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J48">
+  <autoFilter ref="A4:J50">
     <filterColumn colId="8" hiddenButton="0" showButton="1">
       <filters blank="1"/>
     </filterColumn>
@@ -2471,7 +2547,7 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I5:I48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:I50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Corriger,Corriger plus tard,Ne pas corriger,A decider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>